<commit_message>
Import product listing to /us/hcpportal
The product listing page moved from /us/product to /us/hcpportal; map the
import output path so re-running the importer writes the new location.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-product.report.xlsx
+++ b/tools/importer/reports/import-product.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="39">
   <si>
     <t>_reportFile</t>
   </si>
@@ -73,7 +73,7 @@
     <t>contact-us</t>
   </si>
   <si>
-    <t>2026-10-05T14:54:53.678Z</t>
+    <t>2026-10-05T14:56:25.891Z</t>
   </si>
   <si>
     <t>Contact Lupin US | Get in Touch with Our Team</t>
@@ -82,22 +82,52 @@
     <t>https://www.lupin.com/US/contact-us</t>
   </si>
   <si>
+    <t>us/hcpportal.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","cards-product","cards-link-tile","cards-link-tile"]</t>
+  </si>
+  <si>
+    <t>us/hcpportal</t>
+  </si>
+  <si>
+    <t>product</t>
+  </si>
+  <si>
+    <t>2026-10-05T18:14:40.021Z</t>
+  </si>
+  <si>
+    <t>Explore Our Products | Quality Medicines for Better Health.</t>
+  </si>
+  <si>
     <t>us/product.report.json</t>
   </si>
   <si>
-    <t>["hero-banner","cards-product","cards-link-tile","cards-link-tile"]</t>
-  </si>
-  <si>
     <t>us/product</t>
   </si>
   <si>
-    <t>product</t>
-  </si>
-  <si>
     <t>2026-10-05T14:55:04.507Z</t>
   </si>
   <si>
-    <t>Explore Our Products | Quality Medicines for Better Health.</t>
+    <t>us/product/glycerol-phenylbutyrate-oral-liquid.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","columns-product-detail","tabs-audience","columns-anchor-nav","columns-anchor-nav","hero-green-panel","hero-green-panel","columns-icon-tips","cards-pharmacy","cards-pharmacy","accordion-faq","accordion-faq","columns-cta-banner","columns-cta-banner"]</t>
+  </si>
+  <si>
+    <t>us/product/glycerol-phenylbutyrate-oral-liquid</t>
+  </si>
+  <si>
+    <t>product-detail</t>
+  </si>
+  <si>
+    <t>2026-10-05T17:10:00.610Z</t>
+  </si>
+  <si>
+    <t>Glycerol Phenylbutyrate Oral Liquid</t>
+  </si>
+  <si>
+    <t>https://www.lupin.com/US/product/glycerol-phenylbutyrate-oral-liquid</t>
   </si>
 </sst>
 </file>
@@ -486,17 +516,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="27" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
+    <col min="1" max="2" width="50" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="4" max="4" width="48" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="26" customWidth="1"/>
-    <col min="8" max="8" width="50" customWidth="1"/>
-    <col min="9" max="9" width="37" customWidth="1"/>
+    <col min="8" max="9" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -613,6 +641,64 @@
       </c>
       <c r="I4" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G6" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" t="s">
+        <v>37</v>
+      </c>
+      <c r="I6" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>